<commit_message>
Modification in DB related test cases (Registration)
</commit_message>
<xml_diff>
--- a/testdata/register_user.xlsx
+++ b/testdata/register_user.xlsx
@@ -3,12 +3,12 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SeleniumLearning\DemoQa\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF65457E-DDB0-429F-B009-B09D736158AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FF138D7-2B5C-41DE-9952-A02F057BAE7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{A74BF28C-13B3-448C-A368-528222B83AEA}"/>
   </bookViews>
@@ -17,7 +17,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="27">
   <si>
     <t>hafiz@gmail.com</t>
   </si>
@@ -117,22 +117,12 @@
   </si>
   <si>
     <t>hafiz_ahsan4</t>
-  </si>
-  <si>
-    <t>Test Failed</t>
-  </si>
-  <si>
-    <t>Execution Error</t>
-  </si>
-  <si>
-    <t>Test Passed</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
   <fonts count="5">
     <font>
       <sz val="11"/>
@@ -551,12 +541,12 @@
   <dimension ref="A1:G7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="20.140625"/>
-    <col min="2" max="2" customWidth="true" width="19.0"/>
-    <col min="3" max="3" customWidth="true" width="31.140625"/>
-    <col min="4" max="5" customWidth="true" width="30.85546875"/>
-    <col min="6" max="6" customWidth="true" width="24.85546875"/>
-    <col min="7" max="7" customWidth="true" width="27.140625"/>
+    <col min="1" max="1" width="20.140625" customWidth="1"/>
+    <col min="2" max="2" width="19" customWidth="1"/>
+    <col min="3" max="3" width="31.140625" customWidth="1"/>
+    <col min="4" max="5" width="30.85546875" customWidth="1"/>
+    <col min="6" max="6" width="24.85546875" customWidth="1"/>
+    <col min="7" max="7" width="27.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -583,10 +573,10 @@
       </c>
     </row>
     <row r="2" spans="1:7">
-      <c r="A2" t="s" s="0">
+      <c r="A2" t="s">
         <v>11</v>
       </c>
-      <c r="B2" t="s" s="0">
+      <c r="B2" t="s">
         <v>12</v>
       </c>
       <c r="C2" s="2" t="s">
@@ -598,18 +588,12 @@
       <c r="E2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F2" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G2" t="s" s="0">
-        <v>27</v>
-      </c>
     </row>
     <row r="3" spans="1:7">
-      <c r="A3" t="s" s="0">
+      <c r="A3" t="s">
         <v>13</v>
       </c>
-      <c r="B3" t="s" s="0">
+      <c r="B3" t="s">
         <v>14</v>
       </c>
       <c r="C3" s="2" t="s">
@@ -621,18 +605,12 @@
       <c r="E3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F3" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G3" t="s" s="0">
-        <v>27</v>
-      </c>
     </row>
     <row r="4" spans="1:7">
-      <c r="A4" t="s" s="0">
+      <c r="A4" t="s">
         <v>15</v>
       </c>
-      <c r="B4" t="s" s="0">
+      <c r="B4" t="s">
         <v>16</v>
       </c>
       <c r="C4" s="2" t="s">
@@ -644,18 +622,12 @@
       <c r="E4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F4" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G4" t="s" s="0">
-        <v>27</v>
-      </c>
     </row>
     <row r="5" spans="1:7">
-      <c r="A5" t="s" s="0">
+      <c r="A5" t="s">
         <v>17</v>
       </c>
-      <c r="B5" t="s" s="0">
+      <c r="B5" t="s">
         <v>18</v>
       </c>
       <c r="C5" s="2" t="s">
@@ -667,18 +639,12 @@
       <c r="E5" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F5" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G5" t="s" s="0">
-        <v>27</v>
-      </c>
     </row>
     <row r="6" spans="1:7">
-      <c r="A6" t="s" s="0">
+      <c r="A6" t="s">
         <v>21</v>
       </c>
-      <c r="B6" t="s" s="0">
+      <c r="B6" t="s">
         <v>20</v>
       </c>
       <c r="C6" s="2" t="s">
@@ -690,21 +656,15 @@
       <c r="E6" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F6" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G6" t="s" s="0">
-        <v>27</v>
-      </c>
     </row>
     <row r="7" spans="1:7">
-      <c r="A7" t="s" s="0">
+      <c r="A7" t="s">
         <v>19</v>
       </c>
-      <c r="B7" t="s" s="0">
+      <c r="B7" t="s">
         <v>20</v>
       </c>
-      <c r="C7" t="s" s="0">
+      <c r="C7" t="s">
         <v>0</v>
       </c>
       <c r="D7" s="5" t="s">
@@ -712,12 +672,6 @@
       </c>
       <c r="E7" s="1" t="s">
         <v>3</v>
-      </c>
-      <c r="F7" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G7" t="s" s="0">
-        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>